<commit_message>
tweaks to 1-4 handouts
</commit_message>
<xml_diff>
--- a/handouts/chapter_1_4_handout.xlsx
+++ b/handouts/chapter_1_4_handout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\craigaj\Documents\GitHub\timeseries\handouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC944B35-E5FD-4906-9307-671D58DB5C8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB479EB8-EC4C-47F2-BBD2-04049E53E882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-11055" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
   </bookViews>
@@ -94,9 +94,6 @@
 </t>
   </si>
   <si>
-    <t>Random</t>
-  </si>
-  <si>
     <t xml:space="preserve">Seasonally Adjusted
 </t>
   </si>
@@ -334,10 +331,15 @@
 Centered Moving Average,      , and the Estimated Monthly Additive Effect,</t>
   </si>
   <si>
-    <t>Table 3: Computation of        the Random Component and the Seasonally Adjusted Time Series</t>
-  </si>
-  <si>
     <t>Mean,</t>
+  </si>
+  <si>
+    <t>Table 3: Computation of        the Random Component 
+and the Seasonally Adjusted Time Series</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Random
+</t>
   </si>
 </sst>
 </file>
@@ -410,7 +412,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -481,17 +483,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -591,16 +582,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -610,38 +601,53 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -652,11 +658,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -664,32 +667,17 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1953,8 +1941,8 @@
       <xdr:rowOff>163195</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="320040" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="15" name="TextBox 14">
@@ -2003,7 +1991,7 @@
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" i="1">
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -2045,7 +2033,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="15" name="TextBox 14">
@@ -2170,7 +2158,7 @@
                         <m:sSub>
                           <m:sSubPr>
                             <m:ctrlPr>
-                              <a:rPr lang="en-US" sz="1400" i="1">
+                              <a:rPr lang="en-US" sz="1400" b="0" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
                             </m:ctrlPr>
@@ -2285,8 +2273,8 @@
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="379575" cy="250903"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="17" name="TextBox 16">
@@ -2328,7 +2316,6 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
-              <a:pPr/>
               <a14:m>
                 <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:acc>
@@ -2344,7 +2331,7 @@
                       <m:sSub>
                         <m:sSubPr>
                           <m:ctrlPr>
-                            <a:rPr lang="en-US" sz="1400" i="1">
+                            <a:rPr lang="en-US" sz="1400" b="0" i="1">
                               <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                             </a:rPr>
                           </m:ctrlPr>
@@ -2390,7 +2377,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="17" name="TextBox 16">
@@ -2458,8 +2445,8 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>202565</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>399415</xdr:colOff>
       <xdr:row>77</xdr:row>
       <xdr:rowOff>77470</xdr:rowOff>
     </xdr:from>
@@ -2479,7 +2466,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="1878965" y="15546070"/>
+              <a:off x="2923540" y="15003145"/>
               <a:ext cx="320040" cy="221214"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2558,7 +2545,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="1878965" y="15546070"/>
+              <a:off x="2923540" y="15003145"/>
               <a:ext cx="320040" cy="221214"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2659,7 +2646,7 @@
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" i="1">
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -3169,8 +3156,8 @@
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="320040" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="TextBox 7">
@@ -3219,7 +3206,7 @@
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" i="1">
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -3261,7 +3248,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="TextBox 7">
@@ -3309,6 +3296,151 @@
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
                 <a:t>𝑠 ̅_𝑡</a:t>
+              </a:r>
+              <a:endParaRPr lang="en-US" sz="1400"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>256540</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>210586</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="320040" cy="221214"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="9" name="TextBox 8">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6AEC3097-FCC7-2824-0FCB-A513C9E1F93E}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4342765" y="15688711"/>
+              <a:ext cx="320040" cy="221214"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr/>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑧</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑡</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="en-US" sz="1400"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="9" name="TextBox 8">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6AEC3097-FCC7-2824-0FCB-A513C9E1F93E}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4342765" y="15688711"/>
+              <a:ext cx="320040" cy="221214"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr/>
+              <a:r>
+                <a:rPr lang="en-US" sz="1400" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑧_𝑡</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1400"/>
             </a:p>
@@ -3649,12 +3781,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="45.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="30" t="s">
-        <v>80</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="32"/>
+      <c r="A1" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="35"/>
     </row>
     <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
@@ -3668,796 +3800,796 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="33">
+        <v>3</v>
+      </c>
+      <c r="B3" s="23">
         <v>3034</v>
       </c>
-      <c r="C3" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="34" t="s">
-        <v>78</v>
+      <c r="C3" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="24" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="33">
+        <v>4</v>
+      </c>
+      <c r="B4" s="23">
         <v>2748</v>
       </c>
-      <c r="C4" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D4" s="34" t="s">
-        <v>78</v>
+      <c r="C4" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="33">
+        <v>5</v>
+      </c>
+      <c r="B5" s="23">
         <v>3164</v>
       </c>
-      <c r="C5" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D5" s="34" t="s">
-        <v>78</v>
+      <c r="C5" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D5" s="24" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="33">
+        <v>6</v>
+      </c>
+      <c r="B6" s="23">
         <v>3238</v>
       </c>
-      <c r="C6" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D6" s="34" t="s">
-        <v>78</v>
+      <c r="C6" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="33">
+        <v>7</v>
+      </c>
+      <c r="B7" s="23">
         <v>3416</v>
       </c>
-      <c r="C7" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D7" s="34" t="s">
-        <v>78</v>
+      <c r="C7" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="33">
+        <v>8</v>
+      </c>
+      <c r="B8" s="23">
         <v>3492</v>
       </c>
-      <c r="C8" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D8" s="34" t="s">
-        <v>78</v>
+      <c r="C8" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="33">
+        <v>9</v>
+      </c>
+      <c r="B9" s="23">
         <v>3730</v>
       </c>
-      <c r="C9" s="35">
+      <c r="C9" s="25">
         <v>3351.5833333333335</v>
       </c>
-      <c r="D9" s="37">
+      <c r="D9" s="27">
         <f>IFERROR(B9-C9, "NA")</f>
         <v>378.41666666666652</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="33">
+        <v>10</v>
+      </c>
+      <c r="B10" s="23">
         <v>3409</v>
       </c>
-      <c r="C10" s="35">
+      <c r="C10" s="25">
         <v>3350</v>
       </c>
-      <c r="D10" s="36"/>
+      <c r="D10" s="26"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="33">
+        <v>11</v>
+      </c>
+      <c r="B11" s="23">
         <v>3572</v>
       </c>
-      <c r="C11" s="35">
+      <c r="C11" s="25">
         <v>3343.2083333333335</v>
       </c>
-      <c r="D11" s="36"/>
+      <c r="D11" s="26"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="33">
+        <v>12</v>
+      </c>
+      <c r="B12" s="23">
         <v>3629</v>
       </c>
-      <c r="C12" s="35">
+      <c r="C12" s="25">
         <v>3326.2083333333335</v>
       </c>
-      <c r="D12" s="36"/>
+      <c r="D12" s="26"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="33">
+        <v>13</v>
+      </c>
+      <c r="B13" s="23">
         <v>3408</v>
       </c>
-      <c r="C13" s="35">
+      <c r="C13" s="25">
         <v>3316.5416666666665</v>
       </c>
-      <c r="D13" s="36"/>
+      <c r="D13" s="26"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="33">
+        <v>14</v>
+      </c>
+      <c r="B14" s="23">
         <v>3391</v>
       </c>
-      <c r="C14" s="35">
+      <c r="C14" s="25">
         <v>3318.5833333333335</v>
       </c>
-      <c r="D14" s="36"/>
+      <c r="D14" s="26"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="33">
+        <v>15</v>
+      </c>
+      <c r="B15" s="23">
         <v>3010</v>
       </c>
-      <c r="C15" s="35">
+      <c r="C15" s="25">
         <v>3312.0833333333335</v>
       </c>
-      <c r="D15" s="36"/>
+      <c r="D15" s="26"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="33">
+        <v>16</v>
+      </c>
+      <c r="B16" s="23">
         <v>2734</v>
       </c>
-      <c r="C16" s="35">
+      <c r="C16" s="25">
         <v>3308.0416666666665</v>
       </c>
-      <c r="D16" s="36"/>
+      <c r="D16" s="26"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="33">
+        <v>17</v>
+      </c>
+      <c r="B17" s="23">
         <v>3015</v>
       </c>
-      <c r="C17" s="35">
+      <c r="C17" s="25">
         <v>3311.7083333333335</v>
       </c>
-      <c r="D17" s="36"/>
+      <c r="D17" s="26"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="33">
+        <v>18</v>
+      </c>
+      <c r="B18" s="23">
         <v>2979</v>
       </c>
-      <c r="C18" s="35">
+      <c r="C18" s="25">
         <v>3313.1666666666665</v>
       </c>
-      <c r="D18" s="36"/>
+      <c r="D18" s="26"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="33">
+        <v>19</v>
+      </c>
+      <c r="B19" s="23">
         <v>3443</v>
       </c>
-      <c r="C19" s="35">
+      <c r="C19" s="25">
         <v>3307.75</v>
       </c>
-      <c r="D19" s="36"/>
+      <c r="D19" s="26"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="33">
+        <v>20</v>
+      </c>
+      <c r="B20" s="23">
         <v>3514</v>
       </c>
-      <c r="C20" s="35">
+      <c r="C20" s="25">
         <v>3292.4166666666665</v>
       </c>
-      <c r="D20" s="36"/>
+      <c r="D20" s="26"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="33">
+        <v>21</v>
+      </c>
+      <c r="B21" s="23">
         <v>3552</v>
       </c>
-      <c r="C21" s="35">
+      <c r="C21" s="25">
         <v>3281.0833333333335</v>
       </c>
-      <c r="D21" s="36"/>
+      <c r="D21" s="26"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" s="33">
+        <v>22</v>
+      </c>
+      <c r="B22" s="23">
         <v>3490</v>
       </c>
-      <c r="C22" s="35">
+      <c r="C22" s="25">
         <v>3270.2083333333335</v>
       </c>
-      <c r="D22" s="36"/>
+      <c r="D22" s="26"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="33">
+        <v>23</v>
+      </c>
+      <c r="B23" s="23">
         <v>3579</v>
       </c>
-      <c r="C23" s="35">
+      <c r="C23" s="25">
         <v>3259.4583333333335</v>
       </c>
-      <c r="D23" s="36"/>
+      <c r="D23" s="26"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" s="33">
+        <v>24</v>
+      </c>
+      <c r="B24" s="23">
         <v>3657</v>
       </c>
-      <c r="C24" s="35">
+      <c r="C24" s="25">
         <v>3261.1666666666665</v>
       </c>
-      <c r="D24" s="36"/>
+      <c r="D24" s="26"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" s="33">
+        <v>25</v>
+      </c>
+      <c r="B25" s="23">
         <v>3250</v>
       </c>
-      <c r="C25" s="35">
+      <c r="C25" s="25">
         <v>3264.25</v>
       </c>
-      <c r="D25" s="36"/>
+      <c r="D25" s="26"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" s="33">
+        <v>26</v>
+      </c>
+      <c r="B26" s="23">
         <v>3181</v>
       </c>
-      <c r="C26" s="35">
+      <c r="C26" s="25">
         <v>3260.4583333333335</v>
       </c>
-      <c r="D26" s="36"/>
+      <c r="D26" s="26"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" s="33">
+        <v>27</v>
+      </c>
+      <c r="B27" s="23">
         <v>2948</v>
       </c>
-      <c r="C27" s="35">
+      <c r="C27" s="25">
         <v>3256.7083333333335</v>
       </c>
-      <c r="D27" s="36"/>
+      <c r="D27" s="26"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="33">
+        <v>28</v>
+      </c>
+      <c r="B28" s="23">
         <v>2535</v>
       </c>
-      <c r="C28" s="35">
+      <c r="C28" s="25">
         <v>3262.125</v>
       </c>
-      <c r="D28" s="36"/>
+      <c r="D28" s="26"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="33">
+        <v>29</v>
+      </c>
+      <c r="B29" s="23">
         <v>2956</v>
       </c>
-      <c r="C29" s="35">
+      <c r="C29" s="25">
         <v>3267.0833333333335</v>
       </c>
-      <c r="D29" s="36"/>
+      <c r="D29" s="26"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="33">
+        <v>30</v>
+      </c>
+      <c r="B30" s="23">
         <v>3079</v>
       </c>
-      <c r="C30" s="35">
+      <c r="C30" s="25">
         <v>3259.2916666666665</v>
       </c>
-      <c r="D30" s="36"/>
+      <c r="D30" s="26"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B31" s="33">
+        <v>31</v>
+      </c>
+      <c r="B31" s="23">
         <v>3417</v>
       </c>
-      <c r="C31" s="35">
+      <c r="C31" s="25">
         <v>3254</v>
       </c>
-      <c r="D31" s="36"/>
+      <c r="D31" s="26"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" s="33">
+        <v>32</v>
+      </c>
+      <c r="B32" s="23">
         <v>3449</v>
       </c>
-      <c r="C32" s="35">
+      <c r="C32" s="25">
         <v>3256.9583333333335</v>
       </c>
-      <c r="D32" s="36"/>
+      <c r="D32" s="26"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B33" s="33">
+        <v>33</v>
+      </c>
+      <c r="B33" s="23">
         <v>3527</v>
       </c>
-      <c r="C33" s="35">
+      <c r="C33" s="25">
         <v>3256.7083333333335</v>
       </c>
-      <c r="D33" s="36"/>
+      <c r="D33" s="26"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B34" s="33">
+        <v>34</v>
+      </c>
+      <c r="B34" s="23">
         <v>3645</v>
       </c>
-      <c r="C34" s="35">
+      <c r="C34" s="25">
         <v>3269</v>
       </c>
-      <c r="D34" s="36"/>
+      <c r="D34" s="26"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B35" s="33">
+        <v>35</v>
+      </c>
+      <c r="B35" s="23">
         <v>3543</v>
       </c>
-      <c r="C35" s="35">
+      <c r="C35" s="25">
         <v>3279.0833333333335</v>
       </c>
-      <c r="D35" s="36"/>
+      <c r="D35" s="26"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B36" s="33">
+        <v>36</v>
+      </c>
+      <c r="B36" s="23">
         <v>3506</v>
       </c>
-      <c r="C36" s="35">
+      <c r="C36" s="25">
         <v>3252.8333333333335</v>
       </c>
-      <c r="D36" s="36"/>
+      <c r="D36" s="26"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B37" s="33">
+        <v>37</v>
+      </c>
+      <c r="B37" s="23">
         <v>3274</v>
       </c>
-      <c r="C37" s="35">
+      <c r="C37" s="25">
         <v>3228.0416666666665</v>
       </c>
-      <c r="D37" s="36"/>
+      <c r="D37" s="26"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B38" s="33">
+        <v>38</v>
+      </c>
+      <c r="B38" s="23">
         <v>3228</v>
       </c>
-      <c r="C38" s="35">
+      <c r="C38" s="25">
         <v>3248.2083333333335</v>
       </c>
-      <c r="D38" s="36"/>
+      <c r="D38" s="26"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B39" s="33">
+        <v>39</v>
+      </c>
+      <c r="B39" s="23">
         <v>2895</v>
       </c>
-      <c r="C39" s="35">
+      <c r="C39" s="25">
         <v>3294.2916666666665</v>
       </c>
-      <c r="D39" s="36"/>
+      <c r="D39" s="26"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B40" s="33">
+        <v>40</v>
+      </c>
+      <c r="B40" s="23">
         <v>2883</v>
       </c>
-      <c r="C40" s="35">
+      <c r="C40" s="25">
         <v>3340.3333333333335</v>
       </c>
-      <c r="D40" s="36"/>
+      <c r="D40" s="26"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B41" s="33">
+        <v>41</v>
+      </c>
+      <c r="B41" s="23">
         <v>2850</v>
       </c>
-      <c r="C41" s="35">
+      <c r="C41" s="25">
         <v>3384.6666666666665</v>
       </c>
-      <c r="D41" s="36"/>
+      <c r="D41" s="26"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B42" s="33">
+        <v>42</v>
+      </c>
+      <c r="B42" s="23">
         <v>2555</v>
       </c>
-      <c r="C42" s="35">
+      <c r="C42" s="25">
         <v>3433.5416666666665</v>
       </c>
-      <c r="D42" s="36"/>
+      <c r="D42" s="26"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B43" s="33">
+        <v>43</v>
+      </c>
+      <c r="B43" s="23">
         <v>3346</v>
       </c>
-      <c r="C43" s="35">
+      <c r="C43" s="25">
         <v>3481.2916666666665</v>
       </c>
-      <c r="D43" s="36"/>
+      <c r="D43" s="26"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B44" s="33">
+        <v>44</v>
+      </c>
+      <c r="B44" s="23">
         <v>4004</v>
       </c>
-      <c r="C44" s="35">
+      <c r="C44" s="25">
         <v>3514.8333333333335</v>
       </c>
-      <c r="D44" s="36"/>
+      <c r="D44" s="26"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B45" s="33">
+        <v>45</v>
+      </c>
+      <c r="B45" s="23">
         <v>4078</v>
       </c>
-      <c r="C45" s="35">
+      <c r="C45" s="25">
         <v>3549.875</v>
       </c>
-      <c r="D45" s="36"/>
+      <c r="D45" s="26"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B46" s="33">
+        <v>46</v>
+      </c>
+      <c r="B46" s="23">
         <v>4199</v>
       </c>
-      <c r="C46" s="35">
+      <c r="C46" s="25">
         <v>3567.7083333333335</v>
       </c>
-      <c r="D46" s="36"/>
+      <c r="D46" s="26"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B47" s="33">
+        <v>47</v>
+      </c>
+      <c r="B47" s="23">
         <v>4053</v>
       </c>
-      <c r="C47" s="35">
+      <c r="C47" s="25">
         <v>3590.6666666666665</v>
       </c>
-      <c r="D47" s="36"/>
+      <c r="D47" s="26"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B48" s="33">
+        <v>48</v>
+      </c>
+      <c r="B48" s="23">
         <v>4169</v>
       </c>
-      <c r="C48" s="35">
+      <c r="C48" s="25">
         <v>3672.125</v>
       </c>
-      <c r="D48" s="36"/>
+      <c r="D48" s="26"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B49" s="33">
+        <v>49</v>
+      </c>
+      <c r="B49" s="23">
         <v>3757</v>
       </c>
-      <c r="C49" s="35">
+      <c r="C49" s="25">
         <v>3758.1666666666665</v>
       </c>
-      <c r="D49" s="36"/>
+      <c r="D49" s="26"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B50" s="33">
+        <v>50</v>
+      </c>
+      <c r="B50" s="23">
         <v>3550</v>
       </c>
-      <c r="C50" s="35">
+      <c r="C50" s="25">
         <v>3793.7916666666665</v>
       </c>
-      <c r="D50" s="36"/>
+      <c r="D50" s="26"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B51" s="33">
+        <v>51</v>
+      </c>
+      <c r="B51" s="23">
         <v>3414</v>
       </c>
-      <c r="C51" s="35">
+      <c r="C51" s="25">
         <v>3804.8333333333335</v>
       </c>
-      <c r="D51" s="36"/>
+      <c r="D51" s="26"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B52" s="33">
+        <v>52</v>
+      </c>
+      <c r="B52" s="23">
         <v>2792</v>
       </c>
-      <c r="C52" s="35">
+      <c r="C52" s="25">
         <v>3816.625</v>
       </c>
-      <c r="D52" s="36"/>
+      <c r="D52" s="26"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B53" s="33">
+        <v>53</v>
+      </c>
+      <c r="B53" s="23">
         <v>3492</v>
       </c>
-      <c r="C53" s="35">
+      <c r="C53" s="25">
         <v>3830.9583333333335</v>
       </c>
-      <c r="D53" s="36"/>
+      <c r="D53" s="26"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B54" s="33">
+        <v>54</v>
+      </c>
+      <c r="B54" s="23">
         <v>3868</v>
       </c>
-      <c r="C54" s="35">
+      <c r="C54" s="25">
         <v>3853.2916666666665</v>
       </c>
-      <c r="D54" s="36"/>
+      <c r="D54" s="26"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B55" s="33">
+        <v>55</v>
+      </c>
+      <c r="B55" s="23">
         <v>4098</v>
       </c>
-      <c r="C55" s="35">
+      <c r="C55" s="25">
         <v>3875.5</v>
       </c>
-      <c r="D55" s="36"/>
+      <c r="D55" s="26"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B56" s="33">
+        <v>56</v>
+      </c>
+      <c r="B56" s="23">
         <v>4107</v>
       </c>
-      <c r="C56" s="35">
+      <c r="C56" s="25">
         <v>3899.8333333333335</v>
       </c>
-      <c r="D56" s="36"/>
+      <c r="D56" s="26"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B57" s="33">
+        <v>57</v>
+      </c>
+      <c r="B57" s="23">
         <v>4240</v>
       </c>
-      <c r="C57" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D57" s="36"/>
+      <c r="C57" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D57" s="26"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B58" s="33">
+        <v>58</v>
+      </c>
+      <c r="B58" s="23">
         <v>4320</v>
       </c>
-      <c r="C58" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D58" s="36"/>
+      <c r="C58" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D58" s="26"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B59" s="33">
+        <v>59</v>
+      </c>
+      <c r="B59" s="23">
         <v>4276</v>
       </c>
-      <c r="C59" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D59" s="36"/>
+      <c r="C59" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D59" s="26"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B60" s="33">
+        <v>60</v>
+      </c>
+      <c r="B60" s="23">
         <v>4482</v>
       </c>
-      <c r="C60" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D60" s="36"/>
+      <c r="C60" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D60" s="26"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B61" s="33">
+        <v>61</v>
+      </c>
+      <c r="B61" s="23">
         <v>3977</v>
       </c>
-      <c r="C61" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D61" s="36"/>
+      <c r="C61" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D61" s="26"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B62" s="38">
+        <v>62</v>
+      </c>
+      <c r="B62" s="28">
         <v>3914</v>
       </c>
-      <c r="C62" s="38" t="s">
+      <c r="C62" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D62" s="26"/>
+    </row>
+    <row r="66" spans="1:14" ht="34.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A66" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="D62" s="36"/>
-    </row>
-    <row r="66" spans="1:14" ht="34.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="28" t="s">
-        <v>79</v>
-      </c>
-      <c r="B66" s="29"/>
-      <c r="C66" s="29"/>
-      <c r="D66" s="29"/>
-      <c r="E66" s="29"/>
-      <c r="F66" s="29"/>
-      <c r="G66" s="29"/>
-      <c r="H66" s="29"/>
-      <c r="I66" s="29"/>
-      <c r="J66" s="29"/>
-      <c r="K66" s="29"/>
-      <c r="L66" s="29"/>
-      <c r="M66" s="29"/>
+      <c r="B66" s="37"/>
+      <c r="C66" s="37"/>
+      <c r="D66" s="37"/>
+      <c r="E66" s="37"/>
+      <c r="F66" s="37"/>
+      <c r="G66" s="37"/>
+      <c r="H66" s="37"/>
+      <c r="I66" s="37"/>
+      <c r="J66" s="37"/>
+      <c r="K66" s="37"/>
+      <c r="L66" s="37"/>
+      <c r="M66" s="37"/>
       <c r="N66" s="2"/>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A67" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="B67" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="B67" s="16" t="s">
+      <c r="C67" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="C67" s="16" t="s">
+      <c r="D67" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="D67" s="16" t="s">
+      <c r="E67" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="E67" s="16" t="s">
+      <c r="F67" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="F67" s="16" t="s">
+      <c r="G67" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="G67" s="16" t="s">
+      <c r="H67" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="H67" s="16" t="s">
+      <c r="I67" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="I67" s="16" t="s">
+      <c r="J67" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="J67" s="16" t="s">
+      <c r="K67" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="K67" s="16" t="s">
+      <c r="L67" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="L67" s="16" t="s">
+      <c r="M67" s="17" t="s">
         <v>75</v>
-      </c>
-      <c r="M67" s="17" t="s">
-        <v>76</v>
       </c>
       <c r="N67" s="5"/>
     </row>
@@ -4465,66 +4597,66 @@
       <c r="A68" s="22">
         <v>2017</v>
       </c>
-      <c r="B68" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="C68" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D68" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="E68" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="F68" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="G68" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="H68" s="36"/>
-      <c r="I68" s="36"/>
-      <c r="J68" s="36"/>
-      <c r="K68" s="36"/>
-      <c r="L68" s="36"/>
-      <c r="M68" s="36"/>
+      <c r="B68" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="C68" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D68" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="E68" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="F68" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="G68" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="H68" s="26"/>
+      <c r="I68" s="26"/>
+      <c r="J68" s="26"/>
+      <c r="K68" s="26"/>
+      <c r="L68" s="26"/>
+      <c r="M68" s="26"/>
       <c r="N68" s="6"/>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A69" s="22">
         <v>2018</v>
       </c>
-      <c r="B69" s="36"/>
-      <c r="C69" s="36"/>
-      <c r="D69" s="35">
+      <c r="B69" s="26"/>
+      <c r="C69" s="26"/>
+      <c r="D69" s="25">
         <v>-296.70833333333348</v>
       </c>
-      <c r="E69" s="35">
+      <c r="E69" s="25">
         <v>-334.16666666666652</v>
       </c>
-      <c r="F69" s="35">
+      <c r="F69" s="25">
         <v>135.25</v>
       </c>
-      <c r="G69" s="35">
+      <c r="G69" s="25">
         <v>221.58333333333348</v>
       </c>
-      <c r="H69" s="35">
+      <c r="H69" s="25">
         <v>270.91666666666652</v>
       </c>
-      <c r="I69" s="35">
+      <c r="I69" s="25">
         <v>219.79166666666652</v>
       </c>
-      <c r="J69" s="35">
+      <c r="J69" s="25">
         <v>319.54166666666652</v>
       </c>
-      <c r="K69" s="35">
+      <c r="K69" s="25">
         <v>395.83333333333348</v>
       </c>
-      <c r="L69" s="35">
+      <c r="L69" s="25">
         <v>-14.25</v>
       </c>
-      <c r="M69" s="37">
+      <c r="M69" s="27">
         <v>-79.458333333333485</v>
       </c>
       <c r="N69" s="6"/>
@@ -4533,40 +4665,40 @@
       <c r="A70" s="22">
         <v>2019</v>
       </c>
-      <c r="B70" s="35">
+      <c r="B70" s="25">
         <v>-308.70833333333348</v>
       </c>
-      <c r="C70" s="35">
+      <c r="C70" s="25">
         <v>-727.125</v>
       </c>
-      <c r="D70" s="35">
+      <c r="D70" s="25">
         <v>-311.08333333333348</v>
       </c>
-      <c r="E70" s="35">
+      <c r="E70" s="25">
         <v>-180.29166666666652</v>
       </c>
-      <c r="F70" s="35">
+      <c r="F70" s="25">
         <v>163</v>
       </c>
-      <c r="G70" s="35">
+      <c r="G70" s="25">
         <v>192.04166666666652</v>
       </c>
-      <c r="H70" s="35">
+      <c r="H70" s="25">
         <v>270.29166666666652</v>
       </c>
-      <c r="I70" s="35">
+      <c r="I70" s="25">
         <v>376</v>
       </c>
-      <c r="J70" s="35">
+      <c r="J70" s="25">
         <v>263.91666666666652</v>
       </c>
-      <c r="K70" s="35">
+      <c r="K70" s="25">
         <v>253.16666666666652</v>
       </c>
-      <c r="L70" s="35">
+      <c r="L70" s="25">
         <v>45.958333333333485</v>
       </c>
-      <c r="M70" s="37">
+      <c r="M70" s="27">
         <v>-20.208333333333485</v>
       </c>
       <c r="N70" s="6"/>
@@ -4575,143 +4707,143 @@
       <c r="A71" s="22">
         <v>2020</v>
       </c>
-      <c r="B71" s="35">
+      <c r="B71" s="25">
         <v>-399.29166666666652</v>
       </c>
-      <c r="C71" s="35">
+      <c r="C71" s="25">
         <v>-457.33333333333348</v>
       </c>
-      <c r="D71" s="35">
+      <c r="D71" s="25">
         <v>-534.66666666666652</v>
       </c>
-      <c r="E71" s="35">
+      <c r="E71" s="25">
         <v>-878.54166666666652</v>
       </c>
-      <c r="F71" s="35">
+      <c r="F71" s="25">
         <v>-135.29166666666652</v>
       </c>
-      <c r="G71" s="35">
+      <c r="G71" s="25">
         <v>489.16666666666652</v>
       </c>
-      <c r="H71" s="35">
+      <c r="H71" s="25">
         <v>528.125</v>
       </c>
-      <c r="I71" s="35">
+      <c r="I71" s="25">
         <v>631.29166666666652</v>
       </c>
-      <c r="J71" s="35">
+      <c r="J71" s="25">
         <v>462.33333333333348</v>
       </c>
-      <c r="K71" s="35">
+      <c r="K71" s="25">
         <v>496.875</v>
       </c>
-      <c r="L71" s="35">
+      <c r="L71" s="25">
         <v>-1.1666666666665151</v>
       </c>
-      <c r="M71" s="37">
+      <c r="M71" s="27">
         <v>-243.79166666666652</v>
       </c>
-      <c r="N71" s="23" t="s">
-        <v>77</v>
+      <c r="N71" s="38" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A72" s="22">
         <v>2021</v>
       </c>
-      <c r="B72" s="35">
+      <c r="B72" s="25">
         <v>-390.83333333333348</v>
       </c>
-      <c r="C72" s="35">
+      <c r="C72" s="25">
         <v>-1024.625</v>
       </c>
-      <c r="D72" s="35">
+      <c r="D72" s="25">
         <v>-338.95833333333348</v>
       </c>
-      <c r="E72" s="35">
+      <c r="E72" s="25">
         <v>14.708333333333485</v>
       </c>
-      <c r="F72" s="35">
+      <c r="F72" s="25">
         <v>222.5</v>
       </c>
-      <c r="G72" s="35">
+      <c r="G72" s="25">
         <v>207.16666666666652</v>
       </c>
-      <c r="H72" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="I72" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="J72" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="K72" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="L72" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="M72" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="N72" s="24"/>
+      <c r="H72" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="I72" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="J72" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="K72" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="L72" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="M72" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="N72" s="39"/>
     </row>
     <row r="73" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="B73" s="35">
+        <v>80</v>
+      </c>
+      <c r="B73" s="25">
         <v>-350.22916666666674</v>
       </c>
-      <c r="C73" s="35">
+      <c r="C73" s="25">
         <v>-695.78125</v>
       </c>
-      <c r="D73" s="35">
+      <c r="D73" s="25">
         <v>-370.35416666666674</v>
       </c>
-      <c r="E73" s="36"/>
-      <c r="F73" s="36"/>
-      <c r="G73" s="36"/>
-      <c r="H73" s="36"/>
-      <c r="I73" s="36"/>
-      <c r="J73" s="36"/>
-      <c r="K73" s="36"/>
-      <c r="L73" s="36"/>
-      <c r="M73" s="36"/>
+      <c r="E73" s="26"/>
+      <c r="F73" s="26"/>
+      <c r="G73" s="26"/>
+      <c r="H73" s="26"/>
+      <c r="I73" s="26"/>
+      <c r="J73" s="26"/>
+      <c r="K73" s="26"/>
+      <c r="L73" s="26"/>
+      <c r="M73" s="26"/>
       <c r="N73" s="7">
         <v>-5.0060763888889142</v>
       </c>
     </row>
     <row r="74" spans="1:14" ht="19.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="19"/>
-      <c r="B74" s="40">
+      <c r="B74" s="29">
         <v>-345.22309027777783</v>
       </c>
-      <c r="C74" s="36"/>
-      <c r="D74" s="36"/>
-      <c r="E74" s="36"/>
-      <c r="F74" s="36"/>
-      <c r="G74" s="36"/>
-      <c r="H74" s="36"/>
-      <c r="I74" s="36"/>
-      <c r="J74" s="36"/>
-      <c r="K74" s="36"/>
-      <c r="L74" s="36"/>
-      <c r="M74" s="36"/>
+      <c r="C74" s="26"/>
+      <c r="D74" s="26"/>
+      <c r="E74" s="26"/>
+      <c r="F74" s="26"/>
+      <c r="G74" s="26"/>
+      <c r="H74" s="26"/>
+      <c r="I74" s="26"/>
+      <c r="J74" s="26"/>
+      <c r="K74" s="26"/>
+      <c r="L74" s="26"/>
+      <c r="M74" s="26"/>
       <c r="N74" s="8"/>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.35"/>
     <row r="78" spans="1:14" ht="43.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A78" s="25" t="s">
+      <c r="A78" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="B78" s="26"/>
-      <c r="C78" s="26"/>
-      <c r="D78" s="26"/>
-      <c r="E78" s="26"/>
-      <c r="F78" s="26"/>
-      <c r="G78" s="27"/>
+      <c r="B78" s="31"/>
+      <c r="C78" s="31"/>
+      <c r="D78" s="31"/>
+      <c r="E78" s="31"/>
+      <c r="F78" s="31"/>
+      <c r="G78" s="32"/>
     </row>
     <row r="79" spans="1:14" ht="37.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="12" t="s">
@@ -4723,625 +4855,625 @@
       <c r="C79" s="14"/>
       <c r="D79" s="14"/>
       <c r="E79" s="14"/>
-      <c r="F79" s="14" t="s">
+      <c r="F79" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="G79" s="15" t="s">
         <v>2</v>
-      </c>
-      <c r="G79" s="15" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B80" s="33">
+        <v>3</v>
+      </c>
+      <c r="B80" s="23">
         <f>B3</f>
         <v>3034</v>
       </c>
-      <c r="C80" s="33" t="str">
+      <c r="C80" s="23" t="str">
         <f t="shared" ref="C80:D80" si="0">C3</f>
         <v>NA</v>
       </c>
-      <c r="D80" s="33" t="str">
-        <f t="shared" si="0"/>
+      <c r="D80" s="24" t="str">
+        <f>IF(LEN(D3)&gt;0,D3,"")</f>
         <v>NA</v>
       </c>
-      <c r="E80" s="36"/>
-      <c r="F80" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="G80" s="36"/>
+      <c r="E80" s="26"/>
+      <c r="F80" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="G80" s="26"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B81" s="33">
+        <v>4</v>
+      </c>
+      <c r="B81" s="23">
         <f t="shared" ref="B81:D96" si="1">B4</f>
         <v>2748</v>
       </c>
-      <c r="C81" s="33" t="str">
+      <c r="C81" s="23" t="str">
         <f t="shared" si="1"/>
         <v>NA</v>
       </c>
-      <c r="D81" s="37" t="str">
+      <c r="D81" s="24" t="str">
+        <f t="shared" ref="D81:D139" si="2">IF(LEN(D4)&gt;0,D4,"")</f>
+        <v>NA</v>
+      </c>
+      <c r="E81" s="26"/>
+      <c r="F81" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="G81" s="26"/>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A82" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B82" s="23">
+        <f t="shared" si="1"/>
+        <v>3164</v>
+      </c>
+      <c r="C82" s="23" t="str">
         <f t="shared" si="1"/>
         <v>NA</v>
       </c>
-      <c r="E81" s="36"/>
-      <c r="F81" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="G81" s="36"/>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A82" s="3" t="s">
+      <c r="D82" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v>NA</v>
+      </c>
+      <c r="E82" s="26"/>
+      <c r="F82" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="G82" s="26"/>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A83" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B82" s="33">
+      <c r="B83" s="23">
         <f t="shared" si="1"/>
-        <v>3164</v>
-      </c>
-      <c r="C82" s="33" t="str">
+        <v>3238</v>
+      </c>
+      <c r="C83" s="23" t="str">
         <f t="shared" si="1"/>
         <v>NA</v>
       </c>
-      <c r="D82" s="37" t="str">
+      <c r="D83" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v>NA</v>
+      </c>
+      <c r="E83" s="26"/>
+      <c r="F83" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="G83" s="26"/>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A84" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B84" s="23">
+        <f t="shared" si="1"/>
+        <v>3416</v>
+      </c>
+      <c r="C84" s="23" t="str">
         <f t="shared" si="1"/>
         <v>NA</v>
       </c>
-      <c r="E82" s="36"/>
-      <c r="F82" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="G82" s="36"/>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A83" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B83" s="33">
+      <c r="D84" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v>NA</v>
+      </c>
+      <c r="E84" s="26"/>
+      <c r="F84" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="G84" s="26"/>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A85" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B85" s="23">
         <f t="shared" si="1"/>
-        <v>3238</v>
-      </c>
-      <c r="C83" s="33" t="str">
+        <v>3492</v>
+      </c>
+      <c r="C85" s="23" t="str">
         <f t="shared" si="1"/>
         <v>NA</v>
       </c>
-      <c r="D83" s="37" t="str">
-        <f t="shared" si="1"/>
+      <c r="D85" s="24" t="str">
+        <f t="shared" si="2"/>
         <v>NA</v>
       </c>
-      <c r="E83" s="36"/>
-      <c r="F83" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="G83" s="36"/>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A84" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B84" s="33">
-        <f t="shared" si="1"/>
-        <v>3416</v>
-      </c>
-      <c r="C84" s="33" t="str">
-        <f t="shared" si="1"/>
-        <v>NA</v>
-      </c>
-      <c r="D84" s="37" t="str">
-        <f t="shared" si="1"/>
-        <v>NA</v>
-      </c>
-      <c r="E84" s="36"/>
-      <c r="F84" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="G84" s="36"/>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A85" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B85" s="33">
-        <f t="shared" si="1"/>
-        <v>3492</v>
-      </c>
-      <c r="C85" s="33" t="str">
-        <f t="shared" si="1"/>
-        <v>NA</v>
-      </c>
-      <c r="D85" s="37" t="str">
-        <f t="shared" si="1"/>
-        <v>NA</v>
-      </c>
-      <c r="E85" s="36"/>
-      <c r="F85" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="G85" s="36"/>
+      <c r="E85" s="26"/>
+      <c r="F85" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="G85" s="26"/>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B86" s="33">
+        <v>9</v>
+      </c>
+      <c r="B86" s="23">
         <f t="shared" si="1"/>
         <v>3730</v>
       </c>
-      <c r="C86" s="35">
+      <c r="C86" s="25">
         <f t="shared" si="1"/>
         <v>3351.5833333333335</v>
       </c>
-      <c r="D86" s="37">
-        <f t="shared" si="1"/>
+      <c r="D86" s="27">
+        <f t="shared" si="2"/>
         <v>378.41666666666652</v>
       </c>
-      <c r="E86" s="36"/>
-      <c r="F86" s="36"/>
-      <c r="G86" s="36"/>
+      <c r="E86" s="26"/>
+      <c r="F86" s="26"/>
+      <c r="G86" s="26"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B87" s="33">
+        <v>10</v>
+      </c>
+      <c r="B87" s="23">
         <f t="shared" si="1"/>
         <v>3409</v>
       </c>
-      <c r="C87" s="35">
+      <c r="C87" s="25">
         <f t="shared" si="1"/>
         <v>3350</v>
       </c>
-      <c r="D87" s="37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E87" s="36"/>
-      <c r="F87" s="36"/>
-      <c r="G87" s="36"/>
+      <c r="D87" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E87" s="26"/>
+      <c r="F87" s="26"/>
+      <c r="G87" s="26"/>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B88" s="33">
+        <v>11</v>
+      </c>
+      <c r="B88" s="23">
         <f t="shared" si="1"/>
         <v>3572</v>
       </c>
-      <c r="C88" s="35">
+      <c r="C88" s="25">
         <f t="shared" si="1"/>
         <v>3343.2083333333335</v>
       </c>
-      <c r="D88" s="37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E88" s="36"/>
-      <c r="F88" s="36"/>
-      <c r="G88" s="36"/>
+      <c r="D88" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E88" s="26"/>
+      <c r="F88" s="26"/>
+      <c r="G88" s="26"/>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B89" s="33">
+        <v>12</v>
+      </c>
+      <c r="B89" s="23">
         <f t="shared" si="1"/>
         <v>3629</v>
       </c>
-      <c r="C89" s="35">
+      <c r="C89" s="25">
         <f t="shared" si="1"/>
         <v>3326.2083333333335</v>
       </c>
-      <c r="D89" s="37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E89" s="36"/>
-      <c r="F89" s="36"/>
-      <c r="G89" s="36"/>
+      <c r="D89" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E89" s="26"/>
+      <c r="F89" s="26"/>
+      <c r="G89" s="26"/>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B90" s="33">
+        <v>13</v>
+      </c>
+      <c r="B90" s="23">
         <f t="shared" si="1"/>
         <v>3408</v>
       </c>
-      <c r="C90" s="35">
+      <c r="C90" s="25">
         <f t="shared" si="1"/>
         <v>3316.5416666666665</v>
       </c>
-      <c r="D90" s="37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E90" s="36"/>
-      <c r="F90" s="36"/>
-      <c r="G90" s="36"/>
+      <c r="D90" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E90" s="26"/>
+      <c r="F90" s="26"/>
+      <c r="G90" s="26"/>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B91" s="33">
+        <v>14</v>
+      </c>
+      <c r="B91" s="23">
         <f t="shared" si="1"/>
         <v>3391</v>
       </c>
-      <c r="C91" s="35">
+      <c r="C91" s="25">
         <f t="shared" si="1"/>
         <v>3318.5833333333335</v>
       </c>
-      <c r="D91" s="37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E91" s="36"/>
-      <c r="F91" s="36"/>
-      <c r="G91" s="36"/>
+      <c r="D91" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E91" s="26"/>
+      <c r="F91" s="26"/>
+      <c r="G91" s="26"/>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B92" s="33">
+        <v>15</v>
+      </c>
+      <c r="B92" s="23">
         <f t="shared" si="1"/>
         <v>3010</v>
       </c>
-      <c r="C92" s="35">
+      <c r="C92" s="25">
         <f t="shared" si="1"/>
         <v>3312.0833333333335</v>
       </c>
-      <c r="D92" s="37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E92" s="36"/>
-      <c r="F92" s="36"/>
-      <c r="G92" s="36"/>
+      <c r="D92" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E92" s="26"/>
+      <c r="F92" s="26"/>
+      <c r="G92" s="26"/>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B93" s="33">
+        <v>16</v>
+      </c>
+      <c r="B93" s="23">
         <f t="shared" si="1"/>
         <v>2734</v>
       </c>
-      <c r="C93" s="35">
+      <c r="C93" s="25">
         <f t="shared" si="1"/>
         <v>3308.0416666666665</v>
       </c>
-      <c r="D93" s="37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E93" s="36"/>
-      <c r="F93" s="36"/>
-      <c r="G93" s="36"/>
+      <c r="D93" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E93" s="26"/>
+      <c r="F93" s="26"/>
+      <c r="G93" s="26"/>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B94" s="33">
+        <v>17</v>
+      </c>
+      <c r="B94" s="23">
         <f t="shared" si="1"/>
         <v>3015</v>
       </c>
-      <c r="C94" s="35">
+      <c r="C94" s="25">
         <f t="shared" si="1"/>
         <v>3311.7083333333335</v>
       </c>
-      <c r="D94" s="37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E94" s="36"/>
-      <c r="F94" s="36"/>
-      <c r="G94" s="36"/>
+      <c r="D94" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E94" s="26"/>
+      <c r="F94" s="26"/>
+      <c r="G94" s="26"/>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B95" s="33">
+        <v>18</v>
+      </c>
+      <c r="B95" s="23">
         <f t="shared" si="1"/>
         <v>2979</v>
       </c>
-      <c r="C95" s="35">
+      <c r="C95" s="25">
         <f t="shared" si="1"/>
         <v>3313.1666666666665</v>
       </c>
-      <c r="D95" s="37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E95" s="36"/>
-      <c r="F95" s="36"/>
-      <c r="G95" s="36"/>
+      <c r="D95" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E95" s="26"/>
+      <c r="F95" s="26"/>
+      <c r="G95" s="26"/>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B96" s="33">
+        <v>19</v>
+      </c>
+      <c r="B96" s="23">
         <f t="shared" si="1"/>
         <v>3443</v>
       </c>
-      <c r="C96" s="35">
+      <c r="C96" s="25">
         <f t="shared" si="1"/>
         <v>3307.75</v>
       </c>
-      <c r="D96" s="37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E96" s="36"/>
-      <c r="F96" s="36"/>
-      <c r="G96" s="36"/>
+      <c r="D96" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E96" s="26"/>
+      <c r="F96" s="26"/>
+      <c r="G96" s="26"/>
       <c r="H96" s="1"/>
     </row>
     <row r="97" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A97" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B97" s="33">
-        <f t="shared" ref="B97:D112" si="2">B20</f>
+        <v>20</v>
+      </c>
+      <c r="B97" s="23">
+        <f t="shared" ref="B97:D112" si="3">B20</f>
         <v>3514</v>
       </c>
-      <c r="C97" s="35">
+      <c r="C97" s="25">
+        <f t="shared" si="3"/>
+        <v>3292.4166666666665</v>
+      </c>
+      <c r="D97" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3292.4166666666665</v>
-      </c>
-      <c r="D97" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E97" s="36"/>
-      <c r="F97" s="36"/>
-      <c r="G97" s="36"/>
+        <v/>
+      </c>
+      <c r="E97" s="26"/>
+      <c r="F97" s="26"/>
+      <c r="G97" s="26"/>
     </row>
     <row r="98" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A98" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B98" s="33">
+        <v>21</v>
+      </c>
+      <c r="B98" s="23">
+        <f t="shared" si="3"/>
+        <v>3552</v>
+      </c>
+      <c r="C98" s="25">
+        <f t="shared" si="3"/>
+        <v>3281.0833333333335</v>
+      </c>
+      <c r="D98" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3552</v>
-      </c>
-      <c r="C98" s="35">
-        <f t="shared" si="2"/>
-        <v>3281.0833333333335</v>
-      </c>
-      <c r="D98" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E98" s="36"/>
-      <c r="F98" s="36"/>
-      <c r="G98" s="36"/>
+        <v/>
+      </c>
+      <c r="E98" s="26"/>
+      <c r="F98" s="26"/>
+      <c r="G98" s="26"/>
     </row>
     <row r="99" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A99" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B99" s="33">
+        <v>22</v>
+      </c>
+      <c r="B99" s="23">
+        <f t="shared" si="3"/>
+        <v>3490</v>
+      </c>
+      <c r="C99" s="25">
+        <f t="shared" si="3"/>
+        <v>3270.2083333333335</v>
+      </c>
+      <c r="D99" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3490</v>
-      </c>
-      <c r="C99" s="35">
-        <f t="shared" si="2"/>
-        <v>3270.2083333333335</v>
-      </c>
-      <c r="D99" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E99" s="36"/>
-      <c r="F99" s="36"/>
-      <c r="G99" s="36"/>
+        <v/>
+      </c>
+      <c r="E99" s="26"/>
+      <c r="F99" s="26"/>
+      <c r="G99" s="26"/>
     </row>
     <row r="100" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A100" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B100" s="33">
+        <v>23</v>
+      </c>
+      <c r="B100" s="23">
+        <f t="shared" si="3"/>
+        <v>3579</v>
+      </c>
+      <c r="C100" s="25">
+        <f t="shared" si="3"/>
+        <v>3259.4583333333335</v>
+      </c>
+      <c r="D100" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3579</v>
-      </c>
-      <c r="C100" s="35">
-        <f t="shared" si="2"/>
-        <v>3259.4583333333335</v>
-      </c>
-      <c r="D100" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E100" s="36"/>
-      <c r="F100" s="36"/>
-      <c r="G100" s="36"/>
+        <v/>
+      </c>
+      <c r="E100" s="26"/>
+      <c r="F100" s="26"/>
+      <c r="G100" s="26"/>
     </row>
     <row r="101" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A101" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B101" s="33">
+        <v>24</v>
+      </c>
+      <c r="B101" s="23">
+        <f t="shared" si="3"/>
+        <v>3657</v>
+      </c>
+      <c r="C101" s="25">
+        <f t="shared" si="3"/>
+        <v>3261.1666666666665</v>
+      </c>
+      <c r="D101" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3657</v>
-      </c>
-      <c r="C101" s="35">
-        <f t="shared" si="2"/>
-        <v>3261.1666666666665</v>
-      </c>
-      <c r="D101" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E101" s="36"/>
-      <c r="F101" s="36"/>
-      <c r="G101" s="36"/>
+        <v/>
+      </c>
+      <c r="E101" s="26"/>
+      <c r="F101" s="26"/>
+      <c r="G101" s="26"/>
     </row>
     <row r="102" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A102" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B102" s="33">
+        <v>25</v>
+      </c>
+      <c r="B102" s="23">
+        <f t="shared" si="3"/>
+        <v>3250</v>
+      </c>
+      <c r="C102" s="25">
+        <f t="shared" si="3"/>
+        <v>3264.25</v>
+      </c>
+      <c r="D102" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3250</v>
-      </c>
-      <c r="C102" s="35">
-        <f t="shared" si="2"/>
-        <v>3264.25</v>
-      </c>
-      <c r="D102" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E102" s="36"/>
-      <c r="F102" s="36"/>
-      <c r="G102" s="36"/>
+        <v/>
+      </c>
+      <c r="E102" s="26"/>
+      <c r="F102" s="26"/>
+      <c r="G102" s="26"/>
     </row>
     <row r="103" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A103" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B103" s="33">
+        <v>26</v>
+      </c>
+      <c r="B103" s="23">
+        <f t="shared" si="3"/>
+        <v>3181</v>
+      </c>
+      <c r="C103" s="25">
+        <f t="shared" si="3"/>
+        <v>3260.4583333333335</v>
+      </c>
+      <c r="D103" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3181</v>
-      </c>
-      <c r="C103" s="35">
-        <f t="shared" si="2"/>
-        <v>3260.4583333333335</v>
-      </c>
-      <c r="D103" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E103" s="36"/>
-      <c r="F103" s="36"/>
-      <c r="G103" s="36"/>
+        <v/>
+      </c>
+      <c r="E103" s="26"/>
+      <c r="F103" s="26"/>
+      <c r="G103" s="26"/>
     </row>
     <row r="104" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A104" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B104" s="33">
+        <v>27</v>
+      </c>
+      <c r="B104" s="23">
+        <f t="shared" si="3"/>
+        <v>2948</v>
+      </c>
+      <c r="C104" s="25">
+        <f t="shared" si="3"/>
+        <v>3256.7083333333335</v>
+      </c>
+      <c r="D104" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>2948</v>
-      </c>
-      <c r="C104" s="35">
-        <f t="shared" si="2"/>
-        <v>3256.7083333333335</v>
-      </c>
-      <c r="D104" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E104" s="36"/>
-      <c r="F104" s="36"/>
-      <c r="G104" s="36"/>
+        <v/>
+      </c>
+      <c r="E104" s="26"/>
+      <c r="F104" s="26"/>
+      <c r="G104" s="26"/>
     </row>
     <row r="105" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A105" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B105" s="33">
+        <v>28</v>
+      </c>
+      <c r="B105" s="23">
+        <f t="shared" si="3"/>
+        <v>2535</v>
+      </c>
+      <c r="C105" s="25">
+        <f t="shared" si="3"/>
+        <v>3262.125</v>
+      </c>
+      <c r="D105" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>2535</v>
-      </c>
-      <c r="C105" s="35">
-        <f t="shared" si="2"/>
-        <v>3262.125</v>
-      </c>
-      <c r="D105" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E105" s="36"/>
-      <c r="F105" s="36"/>
-      <c r="G105" s="36"/>
+        <v/>
+      </c>
+      <c r="E105" s="26"/>
+      <c r="F105" s="26"/>
+      <c r="G105" s="26"/>
     </row>
     <row r="106" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A106" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B106" s="33">
+        <v>29</v>
+      </c>
+      <c r="B106" s="23">
+        <f t="shared" si="3"/>
+        <v>2956</v>
+      </c>
+      <c r="C106" s="25">
+        <f t="shared" si="3"/>
+        <v>3267.0833333333335</v>
+      </c>
+      <c r="D106" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>2956</v>
-      </c>
-      <c r="C106" s="35">
-        <f t="shared" si="2"/>
-        <v>3267.0833333333335</v>
-      </c>
-      <c r="D106" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E106" s="36"/>
-      <c r="F106" s="36"/>
-      <c r="G106" s="36"/>
+        <v/>
+      </c>
+      <c r="E106" s="26"/>
+      <c r="F106" s="26"/>
+      <c r="G106" s="26"/>
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A107" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B107" s="33">
+        <v>30</v>
+      </c>
+      <c r="B107" s="23">
+        <f t="shared" si="3"/>
+        <v>3079</v>
+      </c>
+      <c r="C107" s="25">
+        <f t="shared" si="3"/>
+        <v>3259.2916666666665</v>
+      </c>
+      <c r="D107" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3079</v>
-      </c>
-      <c r="C107" s="35">
-        <f t="shared" si="2"/>
-        <v>3259.2916666666665</v>
-      </c>
-      <c r="D107" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E107" s="36"/>
-      <c r="F107" s="36"/>
-      <c r="G107" s="36"/>
+        <v/>
+      </c>
+      <c r="E107" s="26"/>
+      <c r="F107" s="26"/>
+      <c r="G107" s="26"/>
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A108" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B108" s="33">
+        <v>31</v>
+      </c>
+      <c r="B108" s="23">
+        <f t="shared" si="3"/>
+        <v>3417</v>
+      </c>
+      <c r="C108" s="25">
+        <f t="shared" si="3"/>
+        <v>3254</v>
+      </c>
+      <c r="D108" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3417</v>
-      </c>
-      <c r="C108" s="35">
-        <f t="shared" si="2"/>
-        <v>3254</v>
-      </c>
-      <c r="D108" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E108" s="36"/>
-      <c r="F108" s="36"/>
-      <c r="G108" s="36"/>
+        <v/>
+      </c>
+      <c r="E108" s="26"/>
+      <c r="F108" s="26"/>
+      <c r="G108" s="26"/>
     </row>
     <row r="109" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A109" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B109" s="33">
+        <v>32</v>
+      </c>
+      <c r="B109" s="23">
+        <f t="shared" si="3"/>
+        <v>3449</v>
+      </c>
+      <c r="C109" s="25">
+        <f t="shared" si="3"/>
+        <v>3256.9583333333335</v>
+      </c>
+      <c r="D109" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3449</v>
-      </c>
-      <c r="C109" s="35">
-        <f t="shared" si="2"/>
-        <v>3256.9583333333335</v>
-      </c>
-      <c r="D109" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E109" s="36"/>
-      <c r="F109" s="36"/>
-      <c r="G109" s="36"/>
+        <v/>
+      </c>
+      <c r="E109" s="26"/>
+      <c r="F109" s="26"/>
+      <c r="G109" s="26"/>
       <c r="H109" s="1"/>
       <c r="I109" s="1"/>
       <c r="J109" s="1"/>
@@ -5351,23 +5483,23 @@
     </row>
     <row r="110" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A110" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B110" s="33">
+        <v>33</v>
+      </c>
+      <c r="B110" s="23">
+        <f t="shared" si="3"/>
+        <v>3527</v>
+      </c>
+      <c r="C110" s="25">
+        <f t="shared" si="3"/>
+        <v>3256.7083333333335</v>
+      </c>
+      <c r="D110" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3527</v>
-      </c>
-      <c r="C110" s="35">
-        <f t="shared" si="2"/>
-        <v>3256.7083333333335</v>
-      </c>
-      <c r="D110" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E110" s="36"/>
-      <c r="F110" s="36"/>
-      <c r="G110" s="36"/>
+        <v/>
+      </c>
+      <c r="E110" s="26"/>
+      <c r="F110" s="26"/>
+      <c r="G110" s="26"/>
       <c r="H110" s="1"/>
       <c r="I110" s="1"/>
       <c r="J110" s="1"/>
@@ -5377,23 +5509,23 @@
     </row>
     <row r="111" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A111" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B111" s="33">
+        <v>34</v>
+      </c>
+      <c r="B111" s="23">
+        <f t="shared" si="3"/>
+        <v>3645</v>
+      </c>
+      <c r="C111" s="25">
+        <f t="shared" si="3"/>
+        <v>3269</v>
+      </c>
+      <c r="D111" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3645</v>
-      </c>
-      <c r="C111" s="35">
-        <f t="shared" si="2"/>
-        <v>3269</v>
-      </c>
-      <c r="D111" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E111" s="36"/>
-      <c r="F111" s="36"/>
-      <c r="G111" s="36"/>
+        <v/>
+      </c>
+      <c r="E111" s="26"/>
+      <c r="F111" s="26"/>
+      <c r="G111" s="26"/>
       <c r="H111" s="1"/>
       <c r="I111" s="1"/>
       <c r="J111" s="1"/>
@@ -5403,23 +5535,23 @@
     </row>
     <row r="112" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A112" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B112" s="33">
+        <v>35</v>
+      </c>
+      <c r="B112" s="23">
+        <f t="shared" si="3"/>
+        <v>3543</v>
+      </c>
+      <c r="C112" s="25">
+        <f t="shared" si="3"/>
+        <v>3279.0833333333335</v>
+      </c>
+      <c r="D112" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>3543</v>
-      </c>
-      <c r="C112" s="35">
-        <f t="shared" si="2"/>
-        <v>3279.0833333333335</v>
-      </c>
-      <c r="D112" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E112" s="36"/>
-      <c r="F112" s="36"/>
-      <c r="G112" s="36"/>
+        <v/>
+      </c>
+      <c r="E112" s="26"/>
+      <c r="F112" s="26"/>
+      <c r="G112" s="26"/>
       <c r="H112" s="1"/>
       <c r="I112" s="1"/>
       <c r="J112" s="1"/>
@@ -5429,43 +5561,43 @@
     </row>
     <row r="113" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A113" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B113" s="33">
-        <f t="shared" ref="B113:D128" si="3">B36</f>
+        <v>36</v>
+      </c>
+      <c r="B113" s="23">
+        <f t="shared" ref="B113:D128" si="4">B36</f>
         <v>3506</v>
       </c>
-      <c r="C113" s="35">
-        <f t="shared" si="3"/>
+      <c r="C113" s="25">
+        <f t="shared" si="4"/>
         <v>3252.8333333333335</v>
       </c>
-      <c r="D113" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E113" s="36"/>
-      <c r="F113" s="36"/>
-      <c r="G113" s="36"/>
+      <c r="D113" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E113" s="26"/>
+      <c r="F113" s="26"/>
+      <c r="G113" s="26"/>
     </row>
     <row r="114" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A114" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B114" s="33">
-        <f t="shared" si="3"/>
+        <v>37</v>
+      </c>
+      <c r="B114" s="23">
+        <f t="shared" si="4"/>
         <v>3274</v>
       </c>
-      <c r="C114" s="35">
-        <f t="shared" si="3"/>
+      <c r="C114" s="25">
+        <f t="shared" si="4"/>
         <v>3228.0416666666665</v>
       </c>
-      <c r="D114" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E114" s="36"/>
-      <c r="F114" s="36"/>
-      <c r="G114" s="36"/>
+      <c r="D114" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E114" s="26"/>
+      <c r="F114" s="26"/>
+      <c r="G114" s="26"/>
       <c r="H114" s="1"/>
       <c r="I114" s="1"/>
       <c r="J114" s="1"/>
@@ -5475,23 +5607,23 @@
     </row>
     <row r="115" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A115" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B115" s="33">
-        <f t="shared" si="3"/>
+        <v>38</v>
+      </c>
+      <c r="B115" s="23">
+        <f t="shared" si="4"/>
         <v>3228</v>
       </c>
-      <c r="C115" s="35">
-        <f t="shared" si="3"/>
+      <c r="C115" s="25">
+        <f t="shared" si="4"/>
         <v>3248.2083333333335</v>
       </c>
-      <c r="D115" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E115" s="36"/>
-      <c r="F115" s="36"/>
-      <c r="G115" s="36"/>
+      <c r="D115" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E115" s="26"/>
+      <c r="F115" s="26"/>
+      <c r="G115" s="26"/>
       <c r="H115" s="1"/>
       <c r="I115" s="1"/>
       <c r="J115" s="1"/>
@@ -5502,483 +5634,483 @@
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A116" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B116" s="33">
-        <f t="shared" si="3"/>
+        <v>39</v>
+      </c>
+      <c r="B116" s="23">
+        <f t="shared" si="4"/>
         <v>2895</v>
       </c>
-      <c r="C116" s="35">
-        <f t="shared" si="3"/>
+      <c r="C116" s="25">
+        <f t="shared" si="4"/>
         <v>3294.2916666666665</v>
       </c>
-      <c r="D116" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E116" s="36"/>
-      <c r="F116" s="36"/>
-      <c r="G116" s="36"/>
+      <c r="D116" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E116" s="26"/>
+      <c r="F116" s="26"/>
+      <c r="G116" s="26"/>
     </row>
     <row r="117" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A117" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B117" s="33">
-        <f t="shared" si="3"/>
+        <v>40</v>
+      </c>
+      <c r="B117" s="23">
+        <f t="shared" si="4"/>
         <v>2883</v>
       </c>
-      <c r="C117" s="35">
-        <f t="shared" si="3"/>
+      <c r="C117" s="25">
+        <f t="shared" si="4"/>
         <v>3340.3333333333335</v>
       </c>
-      <c r="D117" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E117" s="36"/>
-      <c r="F117" s="36"/>
-      <c r="G117" s="36"/>
+      <c r="D117" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E117" s="26"/>
+      <c r="F117" s="26"/>
+      <c r="G117" s="26"/>
     </row>
     <row r="118" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A118" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B118" s="33">
-        <f t="shared" si="3"/>
+        <v>41</v>
+      </c>
+      <c r="B118" s="23">
+        <f t="shared" si="4"/>
         <v>2850</v>
       </c>
-      <c r="C118" s="35">
-        <f t="shared" si="3"/>
+      <c r="C118" s="25">
+        <f t="shared" si="4"/>
         <v>3384.6666666666665</v>
       </c>
-      <c r="D118" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E118" s="36"/>
-      <c r="F118" s="36"/>
-      <c r="G118" s="36"/>
+      <c r="D118" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E118" s="26"/>
+      <c r="F118" s="26"/>
+      <c r="G118" s="26"/>
     </row>
     <row r="119" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A119" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B119" s="33">
-        <f t="shared" si="3"/>
+        <v>42</v>
+      </c>
+      <c r="B119" s="23">
+        <f t="shared" si="4"/>
         <v>2555</v>
       </c>
-      <c r="C119" s="35">
-        <f t="shared" si="3"/>
+      <c r="C119" s="25">
+        <f t="shared" si="4"/>
         <v>3433.5416666666665</v>
       </c>
-      <c r="D119" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E119" s="36"/>
-      <c r="F119" s="36"/>
-      <c r="G119" s="36"/>
+      <c r="D119" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E119" s="26"/>
+      <c r="F119" s="26"/>
+      <c r="G119" s="26"/>
     </row>
     <row r="120" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A120" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B120" s="33">
-        <f t="shared" si="3"/>
+        <v>43</v>
+      </c>
+      <c r="B120" s="23">
+        <f t="shared" si="4"/>
         <v>3346</v>
       </c>
-      <c r="C120" s="35">
-        <f t="shared" si="3"/>
+      <c r="C120" s="25">
+        <f t="shared" si="4"/>
         <v>3481.2916666666665</v>
       </c>
-      <c r="D120" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E120" s="36"/>
-      <c r="F120" s="36"/>
-      <c r="G120" s="36"/>
+      <c r="D120" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E120" s="26"/>
+      <c r="F120" s="26"/>
+      <c r="G120" s="26"/>
     </row>
     <row r="121" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A121" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B121" s="33">
-        <f t="shared" si="3"/>
+        <v>44</v>
+      </c>
+      <c r="B121" s="23">
+        <f t="shared" si="4"/>
         <v>4004</v>
       </c>
-      <c r="C121" s="35">
-        <f t="shared" si="3"/>
+      <c r="C121" s="25">
+        <f t="shared" si="4"/>
         <v>3514.8333333333335</v>
       </c>
-      <c r="D121" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E121" s="36"/>
-      <c r="F121" s="36"/>
-      <c r="G121" s="36"/>
+      <c r="D121" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E121" s="26"/>
+      <c r="F121" s="26"/>
+      <c r="G121" s="26"/>
     </row>
     <row r="122" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A122" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B122" s="33">
-        <f t="shared" si="3"/>
+        <v>45</v>
+      </c>
+      <c r="B122" s="23">
+        <f t="shared" si="4"/>
         <v>4078</v>
       </c>
-      <c r="C122" s="35">
-        <f t="shared" si="3"/>
+      <c r="C122" s="25">
+        <f t="shared" si="4"/>
         <v>3549.875</v>
       </c>
-      <c r="D122" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E122" s="36"/>
-      <c r="F122" s="36"/>
-      <c r="G122" s="36"/>
+      <c r="D122" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E122" s="26"/>
+      <c r="F122" s="26"/>
+      <c r="G122" s="26"/>
     </row>
     <row r="123" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A123" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B123" s="33">
-        <f t="shared" si="3"/>
+        <v>46</v>
+      </c>
+      <c r="B123" s="23">
+        <f t="shared" si="4"/>
         <v>4199</v>
       </c>
-      <c r="C123" s="35">
-        <f t="shared" si="3"/>
+      <c r="C123" s="25">
+        <f t="shared" si="4"/>
         <v>3567.7083333333335</v>
       </c>
-      <c r="D123" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E123" s="36"/>
-      <c r="F123" s="36"/>
-      <c r="G123" s="36"/>
+      <c r="D123" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E123" s="26"/>
+      <c r="F123" s="26"/>
+      <c r="G123" s="26"/>
     </row>
     <row r="124" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A124" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B124" s="33">
-        <f t="shared" si="3"/>
+        <v>47</v>
+      </c>
+      <c r="B124" s="23">
+        <f t="shared" si="4"/>
         <v>4053</v>
       </c>
-      <c r="C124" s="35">
-        <f t="shared" si="3"/>
+      <c r="C124" s="25">
+        <f t="shared" si="4"/>
         <v>3590.6666666666665</v>
       </c>
-      <c r="D124" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E124" s="36"/>
-      <c r="F124" s="36"/>
-      <c r="G124" s="36"/>
+      <c r="D124" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E124" s="26"/>
+      <c r="F124" s="26"/>
+      <c r="G124" s="26"/>
     </row>
     <row r="125" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A125" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B125" s="33">
-        <f t="shared" si="3"/>
+        <v>48</v>
+      </c>
+      <c r="B125" s="23">
+        <f t="shared" si="4"/>
         <v>4169</v>
       </c>
-      <c r="C125" s="35">
-        <f t="shared" si="3"/>
+      <c r="C125" s="25">
+        <f t="shared" si="4"/>
         <v>3672.125</v>
       </c>
-      <c r="D125" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E125" s="36"/>
-      <c r="F125" s="36"/>
-      <c r="G125" s="36"/>
+      <c r="D125" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E125" s="26"/>
+      <c r="F125" s="26"/>
+      <c r="G125" s="26"/>
     </row>
     <row r="126" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A126" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B126" s="33">
-        <f t="shared" si="3"/>
+        <v>49</v>
+      </c>
+      <c r="B126" s="23">
+        <f t="shared" si="4"/>
         <v>3757</v>
       </c>
-      <c r="C126" s="35">
-        <f t="shared" si="3"/>
+      <c r="C126" s="25">
+        <f t="shared" si="4"/>
         <v>3758.1666666666665</v>
       </c>
-      <c r="D126" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E126" s="36"/>
-      <c r="F126" s="36"/>
-      <c r="G126" s="36"/>
+      <c r="D126" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E126" s="26"/>
+      <c r="F126" s="26"/>
+      <c r="G126" s="26"/>
     </row>
     <row r="127" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A127" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B127" s="33">
-        <f t="shared" si="3"/>
+        <v>50</v>
+      </c>
+      <c r="B127" s="23">
+        <f t="shared" si="4"/>
         <v>3550</v>
       </c>
-      <c r="C127" s="35">
-        <f t="shared" si="3"/>
+      <c r="C127" s="25">
+        <f t="shared" si="4"/>
         <v>3793.7916666666665</v>
       </c>
-      <c r="D127" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E127" s="36"/>
-      <c r="F127" s="36"/>
-      <c r="G127" s="36"/>
+      <c r="D127" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E127" s="26"/>
+      <c r="F127" s="26"/>
+      <c r="G127" s="26"/>
     </row>
     <row r="128" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A128" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B128" s="33">
-        <f t="shared" si="3"/>
+        <v>51</v>
+      </c>
+      <c r="B128" s="23">
+        <f t="shared" si="4"/>
         <v>3414</v>
       </c>
-      <c r="C128" s="35">
-        <f t="shared" si="3"/>
+      <c r="C128" s="25">
+        <f t="shared" si="4"/>
         <v>3804.8333333333335</v>
       </c>
-      <c r="D128" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="E128" s="36"/>
-      <c r="F128" s="36"/>
-      <c r="G128" s="36"/>
+      <c r="D128" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E128" s="26"/>
+      <c r="F128" s="26"/>
+      <c r="G128" s="26"/>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A129" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B129" s="33">
-        <f t="shared" ref="B129:D139" si="4">B52</f>
+        <v>52</v>
+      </c>
+      <c r="B129" s="23">
+        <f t="shared" ref="B129:D139" si="5">B52</f>
         <v>2792</v>
       </c>
-      <c r="C129" s="35">
-        <f t="shared" si="4"/>
+      <c r="C129" s="25">
+        <f t="shared" si="5"/>
         <v>3816.625</v>
       </c>
-      <c r="D129" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E129" s="36"/>
-      <c r="F129" s="36"/>
-      <c r="G129" s="36"/>
+      <c r="D129" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E129" s="26"/>
+      <c r="F129" s="26"/>
+      <c r="G129" s="26"/>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A130" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B130" s="33">
-        <f t="shared" si="4"/>
+        <v>53</v>
+      </c>
+      <c r="B130" s="23">
+        <f t="shared" si="5"/>
         <v>3492</v>
       </c>
-      <c r="C130" s="35">
-        <f t="shared" si="4"/>
+      <c r="C130" s="25">
+        <f t="shared" si="5"/>
         <v>3830.9583333333335</v>
       </c>
-      <c r="D130" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E130" s="36"/>
-      <c r="F130" s="36"/>
-      <c r="G130" s="36"/>
+      <c r="D130" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E130" s="26"/>
+      <c r="F130" s="26"/>
+      <c r="G130" s="26"/>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A131" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B131" s="33">
-        <f t="shared" si="4"/>
+        <v>54</v>
+      </c>
+      <c r="B131" s="23">
+        <f t="shared" si="5"/>
         <v>3868</v>
       </c>
-      <c r="C131" s="35">
-        <f t="shared" si="4"/>
+      <c r="C131" s="25">
+        <f t="shared" si="5"/>
         <v>3853.2916666666665</v>
       </c>
-      <c r="D131" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E131" s="36"/>
-      <c r="F131" s="36"/>
-      <c r="G131" s="36"/>
+      <c r="D131" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E131" s="26"/>
+      <c r="F131" s="26"/>
+      <c r="G131" s="26"/>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A132" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B132" s="33">
-        <f t="shared" si="4"/>
+        <v>55</v>
+      </c>
+      <c r="B132" s="23">
+        <f t="shared" si="5"/>
         <v>4098</v>
       </c>
-      <c r="C132" s="35">
-        <f t="shared" si="4"/>
+      <c r="C132" s="25">
+        <f t="shared" si="5"/>
         <v>3875.5</v>
       </c>
-      <c r="D132" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E132" s="36"/>
-      <c r="F132" s="36"/>
-      <c r="G132" s="36"/>
+      <c r="D132" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E132" s="26"/>
+      <c r="F132" s="26"/>
+      <c r="G132" s="26"/>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A133" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B133" s="33">
-        <f t="shared" si="4"/>
+        <v>56</v>
+      </c>
+      <c r="B133" s="23">
+        <f t="shared" si="5"/>
         <v>4107</v>
       </c>
-      <c r="C133" s="35">
-        <f t="shared" si="4"/>
+      <c r="C133" s="25">
+        <f t="shared" si="5"/>
         <v>3899.8333333333335</v>
       </c>
-      <c r="D133" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E133" s="36"/>
-      <c r="F133" s="36"/>
-      <c r="G133" s="36"/>
+      <c r="D133" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E133" s="26"/>
+      <c r="F133" s="26"/>
+      <c r="G133" s="26"/>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A134" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B134" s="33">
-        <f t="shared" si="4"/>
+        <v>57</v>
+      </c>
+      <c r="B134" s="23">
+        <f t="shared" si="5"/>
         <v>4240</v>
       </c>
-      <c r="C134" s="33" t="str">
-        <f t="shared" si="4"/>
+      <c r="C134" s="23" t="str">
+        <f t="shared" si="5"/>
         <v>NA</v>
       </c>
-      <c r="D134" s="34">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E134" s="36"/>
-      <c r="F134" s="36"/>
-      <c r="G134" s="36"/>
+      <c r="D134" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E134" s="26"/>
+      <c r="F134" s="26"/>
+      <c r="G134" s="26"/>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A135" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B135" s="33">
-        <f t="shared" si="4"/>
+        <v>58</v>
+      </c>
+      <c r="B135" s="23">
+        <f t="shared" si="5"/>
         <v>4320</v>
       </c>
-      <c r="C135" s="33" t="str">
-        <f t="shared" si="4"/>
+      <c r="C135" s="23" t="str">
+        <f t="shared" si="5"/>
         <v>NA</v>
       </c>
-      <c r="D135" s="34">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E135" s="36"/>
-      <c r="F135" s="36"/>
-      <c r="G135" s="36"/>
+      <c r="D135" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E135" s="26"/>
+      <c r="F135" s="26"/>
+      <c r="G135" s="26"/>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A136" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B136" s="33">
-        <f t="shared" si="4"/>
+        <v>59</v>
+      </c>
+      <c r="B136" s="23">
+        <f t="shared" si="5"/>
         <v>4276</v>
       </c>
-      <c r="C136" s="33" t="str">
-        <f t="shared" si="4"/>
+      <c r="C136" s="23" t="str">
+        <f t="shared" si="5"/>
         <v>NA</v>
       </c>
-      <c r="D136" s="34">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E136" s="36"/>
-      <c r="F136" s="36"/>
-      <c r="G136" s="36"/>
+      <c r="D136" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E136" s="26"/>
+      <c r="F136" s="26"/>
+      <c r="G136" s="26"/>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A137" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B137" s="33">
-        <f t="shared" si="4"/>
+        <v>60</v>
+      </c>
+      <c r="B137" s="23">
+        <f t="shared" si="5"/>
         <v>4482</v>
       </c>
-      <c r="C137" s="33" t="str">
-        <f t="shared" si="4"/>
+      <c r="C137" s="23" t="str">
+        <f t="shared" si="5"/>
         <v>NA</v>
       </c>
-      <c r="D137" s="34">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E137" s="36"/>
-      <c r="F137" s="36"/>
-      <c r="G137" s="36"/>
+      <c r="D137" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E137" s="26"/>
+      <c r="F137" s="26"/>
+      <c r="G137" s="26"/>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B138" s="33">
-        <f t="shared" si="4"/>
+        <v>61</v>
+      </c>
+      <c r="B138" s="23">
+        <f t="shared" si="5"/>
         <v>3977</v>
       </c>
-      <c r="C138" s="33" t="str">
-        <f t="shared" si="4"/>
+      <c r="C138" s="23" t="str">
+        <f t="shared" si="5"/>
         <v>NA</v>
       </c>
-      <c r="D138" s="34">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E138" s="36"/>
-      <c r="F138" s="36"/>
-      <c r="G138" s="36"/>
+      <c r="D138" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E138" s="26"/>
+      <c r="F138" s="26"/>
+      <c r="G138" s="26"/>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A139" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B139" s="38">
-        <f t="shared" si="4"/>
+        <v>62</v>
+      </c>
+      <c r="B139" s="28">
+        <f t="shared" si="5"/>
         <v>3914</v>
       </c>
-      <c r="C139" s="38" t="str">
-        <f t="shared" si="4"/>
+      <c r="C139" s="28" t="str">
+        <f t="shared" si="5"/>
         <v>NA</v>
       </c>
-      <c r="D139" s="39">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E139" s="36"/>
-      <c r="F139" s="36"/>
-      <c r="G139" s="36"/>
+      <c r="D139" s="26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E139" s="26"/>
+      <c r="F139" s="26"/>
+      <c r="G139" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -5995,12 +6127,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6199,17 +6330,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5E1B631-90B0-4D19-A35E-F8DC8BE167A4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
+    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6234,18 +6375,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5E1B631-90B0-4D19-A35E-F8DC8BE167A4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
-    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>